<commit_message>
Update weekly planning document
Ultraworked with [Sisyphus](https://github.com/code-yeongyu/oh-my-openagent)

Co-authored-by: Sisyphus <clio-agent@sisyphuslabs.ai>
</commit_message>
<xml_diff>
--- a/docs/planning/creador gantt/Planificación semanal actual .xlsx
+++ b/docs/planning/creador gantt/Planificación semanal actual .xlsx
@@ -476,7 +476,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="es-CL"/>
               </a:p>
@@ -587,7 +587,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CL"/>
           </a:p>
@@ -686,7 +686,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CL"/>
           </a:p>
@@ -5342,7 +5342,11 @@
       <c r="B99" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C99" s="29" t="n"/>
+      <c r="C99" s="29" t="inlineStr">
+        <is>
+          <t>FPU habilitada (configENABLE_FPU=1), DMA SPI2 implementado (DMA1 Stream 3/4), WoM interrupt configurado (EXTI9_5_IRQn), CLI extendido (fpu, dma, wom, sensstat, readreg, at, debug), test_suite.c actualizado (8 tests), documentación técnica v1.1.0 actualizada [24 HH]</t>
+        </is>
+      </c>
       <c r="D99" s="1" t="n"/>
       <c r="E99" s="29" t="inlineStr">
         <is>
@@ -5359,7 +5363,7 @@
       </c>
       <c r="H99" s="29" t="inlineStr">
         <is>
-          <t>Adquisición continua: validación de estabilidad 24h [8 HH]</t>
+          <t>Validación pipeline completo 24h en hardware [8 HH]</t>
         </is>
       </c>
       <c r="I99" s="1" t="n"/>
@@ -5388,7 +5392,11 @@
       <c r="B100" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C100" s="29" t="n"/>
+      <c r="C100" s="29" t="inlineStr">
+        <is>
+          <t>Validación de pipeline completo sensor→SD→módem en hardware real [6 HH]</t>
+        </is>
+      </c>
       <c r="D100" s="1" t="n"/>
       <c r="E100" s="29" t="inlineStr">
         <is>
@@ -5434,7 +5442,11 @@
       <c r="B101" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C101" s="29" t="n"/>
+      <c r="C101" s="29" t="inlineStr">
+        <is>
+          <t>Calibración acelerómetro ADXL355: pruebas con referencia [6 HH]</t>
+        </is>
+      </c>
       <c r="D101" s="1" t="n"/>
       <c r="E101" s="29" t="inlineStr">
         <is>
@@ -5451,7 +5463,7 @@
       </c>
       <c r="H101" s="29" t="inlineStr">
         <is>
-          <t>Buffer local: implementación en SD [6 HH]</t>
+          <t>Buffer local SD: implementación y pruebas [6 HH]</t>
         </is>
       </c>
       <c r="I101" s="1" t="n"/>
@@ -5480,7 +5492,11 @@
       <c r="B102" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C102" s="29" t="n"/>
+      <c r="C102" s="29" t="inlineStr">
+        <is>
+          <t>Buffer local SD: diseño arquitectura e implementación inicial [4 HH]</t>
+        </is>
+      </c>
       <c r="D102" s="1" t="n"/>
       <c r="E102" s="29" t="inlineStr">
         <is>
@@ -5493,7 +5509,7 @@
       </c>
       <c r="H102" s="29" t="inlineStr">
         <is>
-          <t>FPU habilitación + pruebas de rendimiento [4 HH]</t>
+          <t>NTP sobre LTE: comandos AT+QNTP + pruebas [4 HH]</t>
         </is>
       </c>
       <c r="I102" s="1" t="n"/>
@@ -5659,7 +5675,11 @@
       <c r="B106" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C106" s="29" t="n"/>
+      <c r="C106" s="29" t="inlineStr">
+        <is>
+          <t>Pipeline completo validado 24h, calibración acelerómetro completada, buffer local SD implementado, NTP LTE integrado [24 HH]</t>
+        </is>
+      </c>
       <c r="D106" s="1" t="n"/>
       <c r="E106" s="29" t="inlineStr">
         <is>
@@ -5705,7 +5725,11 @@
       <c r="B107" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C107" s="29" t="n"/>
+      <c r="C107" s="29" t="inlineStr">
+        <is>
+          <t>Monitoreo baterías Li-Ion: ADC STM32 + temperatura [6 HH]</t>
+        </is>
+      </c>
       <c r="D107" s="1" t="n"/>
       <c r="E107" s="29" t="inlineStr">
         <is>
@@ -5722,7 +5746,7 @@
       </c>
       <c r="H107" s="29" t="inlineStr">
         <is>
-          <t>Sincronización NTP: comandos AT+ Quectel [6 HH]</t>
+          <t>Sincronización NTP: validación en campo [6 HH]</t>
         </is>
       </c>
       <c r="I107" s="1" t="n"/>
@@ -5751,7 +5775,11 @@
       <c r="B108" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C108" s="29" t="n"/>
+      <c r="C108" s="29" t="inlineStr">
+        <is>
+          <t>PCB alimentación: diseño esquemático [8 HH]</t>
+        </is>
+      </c>
       <c r="D108" s="1" t="n"/>
       <c r="E108" s="29" t="inlineStr">
         <is>
@@ -5768,7 +5796,7 @@
       </c>
       <c r="H108" s="29" t="inlineStr">
         <is>
-          <t>Validación banco baterías Li-Ion: capacidad [6 HH]</t>
+          <t>Validación banco baterías Li-Ion: capacidad y ciclos [6 HH]</t>
         </is>
       </c>
       <c r="I108" s="1" t="n"/>
@@ -5797,7 +5825,11 @@
       <c r="B109" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C109" s="29" t="n"/>
+      <c r="C109" s="29" t="inlineStr">
+        <is>
+          <t>Protecciones eléctricas: TVS + Polyswitch [4 HH]</t>
+        </is>
+      </c>
       <c r="D109" s="1" t="n"/>
       <c r="E109" s="29" t="inlineStr">
         <is>
@@ -5810,7 +5842,7 @@
       </c>
       <c r="H109" s="29" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>PCB alimentación: layout y routing [10 HH]</t>
         </is>
       </c>
       <c r="I109" s="1" t="n"/>

</xml_diff>

<commit_message>
fix(upload-pipeline): Modem_PowerOff moved to modem_task + backup registers + GANTT/planning updated
- Modem_PowerOff reubicado a modem_task.c: NRST ahora ocurre DESPUES de queue pop + .DONE
- Backup registers RTC (BKP0R-BKP19R): tracking upload sobrevive NRST/IWDG
- upload_queue_pop(NULL,0) UB fix: NULL guard en strncpy
- Boot scan: skip por backup register + .DONE fallback visible
- .DONE marker: HAL_Delay(50) post f_close para dar tiempo NAND program
- GANTT 2026: fix infinite loop in month iteration
- Planificacion semanal actualizada a Semana 26
</commit_message>
<xml_diff>
--- a/docs/planning/creador gantt/Planificación semanal actual .xlsx
+++ b/docs/planning/creador gantt/Planificación semanal actual .xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3420" yWindow="500" windowWidth="25380" windowHeight="17500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planificación Semanal" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Planificación Semanal" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -381,14 +381,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1200" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -411,8 +411,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+        <a:ln>
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -439,10 +439,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4472C4"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -450,18 +450,18 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -557,8 +557,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -570,9 +570,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -610,7 +610,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -625,9 +625,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -650,8 +650,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill/>
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -662,16 +662,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+          <a:ln>
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -701,10 +701,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -714,7 +714,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>11</col>
@@ -734,9 +734,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -3937,7 +3937,7 @@
       </c>
       <c r="C66" s="18" t="inlineStr">
         <is>
-          <t>Migración de interrupción Wake-on-Motion a NVIC con CMSIS-RTOS v2. Requiere refactorización del manejo de interrupciones del ADXL355 desde el modelo bare-metal al modelo RTOS con event flags. La rutina de interrupción debe señalizar a sensor_task en lugar de manejar datos directamente. [3 HH]</t>
+          <t>Fix residual NRST post-upload por corriente de modem al cerrar TCP</t>
         </is>
       </c>
       <c r="D66" s="1" t="n"/>
@@ -3975,7 +3975,7 @@
       </c>
       <c r="C67" s="18" t="inlineStr">
         <is>
-          <t>Pruebas de compilación cruzada y validación de enlace. Verificar que todas las dependencias entre módulos estén correctamente vinculadas en el nuevo proyecto CMSIS. Resolver posibles errores L6218E (símbolos no resueltos) en la toolchain ARM GCC. [2 HH]</t>
+          <t>NTP sync: ambos servidores fallan, investigar timing AT+QNTP</t>
         </is>
       </c>
       <c r="D67" s="1" t="n"/>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="C68" s="18" t="inlineStr">
         <is>
-          <t>Implementación de script de automatización de flasheo y prueba. Crear script para automatizar flasheo vía OpenOCD y captura de logs seriales para pruebas repetibles. [2 HH]</t>
+          <t>SD mount: primer intento falla (FRESULT=1), retry exitoso</t>
         </is>
       </c>
       <c r="D68" s="1" t="n"/>
@@ -5241,7 +5241,7 @@
       <c r="A97" s="1" t="n"/>
       <c r="B97" s="27" t="inlineStr">
         <is>
-          <t>Semana 25: 16 al 20 Jun 2026 [ACTUAL]</t>
+          <t>Semana 25: 16 al 20 Jun 2026</t>
         </is>
       </c>
       <c r="C97" s="1" t="n"/>
@@ -5344,7 +5344,7 @@
       </c>
       <c r="C99" s="29" t="inlineStr">
         <is>
-          <t>FPU habilitada (configENABLE_FPU=1), DMA SPI2 implementado (DMA1 Stream 3/4), WoM interrupt configurado (EXTI9_5_IRQn), CLI extendido (fpu, dma, wom, sensstat, readreg, at, debug), test_suite.c actualizado (8 tests), documentación técnica v1.1.0 actualizada [24 HH]</t>
+          <t>FPU habilitada, DMA SPI2 implementado, validacion pipeline sensor-&gt;SD-&gt;modem en hardware real [4 HH]</t>
         </is>
       </c>
       <c r="D99" s="1" t="n"/>
@@ -5363,7 +5363,7 @@
       </c>
       <c r="H99" s="29" t="inlineStr">
         <is>
-          <t>Validación pipeline completo 24h en hardware [8 HH]</t>
+          <t>Cola RAM upload implementada (8 slots circulares) [6 HH]</t>
         </is>
       </c>
       <c r="I99" s="1" t="n"/>
@@ -5394,7 +5394,7 @@
       </c>
       <c r="C100" s="29" t="inlineStr">
         <is>
-          <t>Validación de pipeline completo sensor→SD→módem en hardware real [6 HH]</t>
+          <t>Validacion pipeline completo 24h: firmware compilado y flasheado [4 HH]</t>
         </is>
       </c>
       <c r="D100" s="1" t="n"/>
@@ -5413,7 +5413,7 @@
       </c>
       <c r="H100" s="29" t="inlineStr">
         <is>
-          <t>Calibración acelerómetro: pruebas con referencia [6 HH]</t>
+          <t>Backup registers RTC: tracking upload BKP0R-BKP19R [4 HH]</t>
         </is>
       </c>
       <c r="I100" s="1" t="n"/>
@@ -5444,7 +5444,7 @@
       </c>
       <c r="C101" s="29" t="inlineStr">
         <is>
-          <t>Calibración acelerómetro ADXL355: pruebas con referencia [6 HH]</t>
+          <t>Calibracion acelerometro ADXL355: pruebas con referencia [6 HH]</t>
         </is>
       </c>
       <c r="D101" s="1" t="n"/>
@@ -5463,7 +5463,7 @@
       </c>
       <c r="H101" s="29" t="inlineStr">
         <is>
-          <t>Buffer local SD: implementación y pruebas [6 HH]</t>
+          <t>Modem_PowerOff reubicado a modem_task + fix NRST [4 HH]</t>
         </is>
       </c>
       <c r="I101" s="1" t="n"/>
@@ -5494,7 +5494,7 @@
       </c>
       <c r="C102" s="29" t="inlineStr">
         <is>
-          <t>Buffer local SD: diseño arquitectura e implementación inicial [4 HH]</t>
+          <t>Buffer local SD: diseno arquitectura e implementacion inicial [4 HH]</t>
         </is>
       </c>
       <c r="D102" s="1" t="n"/>
@@ -5509,7 +5509,7 @@
       </c>
       <c r="H102" s="29" t="inlineStr">
         <is>
-          <t>NTP sobre LTE: comandos AT+QNTP + pruebas [4 HH]</t>
+          <t>Boot scan + fix UB + upload concurrente [4 HH]</t>
         </is>
       </c>
       <c r="I102" s="1" t="n"/>
@@ -5574,7 +5574,7 @@
       <c r="A104" s="1" t="n"/>
       <c r="B104" s="27" t="inlineStr">
         <is>
-          <t>Semana 26: 23 al 27 Jun 2026</t>
+          <t>Semana 26: 23 al 27 Jun 2026 [ACTUAL]</t>
         </is>
       </c>
       <c r="C104" s="1" t="n"/>
@@ -5677,13 +5677,13 @@
       </c>
       <c r="C106" s="29" t="inlineStr">
         <is>
-          <t>Pipeline completo validado 24h, calibración acelerómetro completada, buffer local SD implementado, NTP LTE integrado [24 HH]</t>
+          <t>Upload pipeline estable: 3 uploads encadenados (TRIG_006/007/008) sin NRST. Backup registers funcionando (BKP0R-BKP19R). Modem_PowerOff reubicado a modem_task. [6 HH]</t>
         </is>
       </c>
       <c r="D106" s="1" t="n"/>
       <c r="E106" s="29" t="inlineStr">
         <is>
-          <t>NTP: integración con Quectel EC25</t>
+          <t>NTP: falla con ambos servidores Google/pool.ntp.org</t>
         </is>
       </c>
       <c r="F106" s="29" t="inlineStr">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="H106" s="29" t="inlineStr">
         <is>
-          <t>Adquisición continua: pruebas extended 48h+ [8 HH]</t>
+          <t>Validacion pipeline 48h: multiple triggers + upload sin NRST [8 HH]</t>
         </is>
       </c>
       <c r="I106" s="1" t="n"/>
@@ -5727,13 +5727,13 @@
       </c>
       <c r="C107" s="29" t="inlineStr">
         <is>
-          <t>Monitoreo baterías Li-Ion: ADC STM32 + temperatura [6 HH]</t>
+          <t>Cola RAM upload 8 slots: implementacion, fix upload_queue_pop(NULL,0) UB, boot scan con skip por backup register. [4 HH]</t>
         </is>
       </c>
       <c r="D107" s="1" t="n"/>
       <c r="E107" s="29" t="inlineStr">
         <is>
-          <t>PCB dedicado alimentación</t>
+          <t>SD mount: falla primer intento, exito en retry</t>
         </is>
       </c>
       <c r="F107" s="29" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="H107" s="29" t="inlineStr">
         <is>
-          <t>Sincronización NTP: validación en campo [6 HH]</t>
+          <t>Fix SD mount retry: investigar causa primer fallo [4 HH]</t>
         </is>
       </c>
       <c r="I107" s="1" t="n"/>
@@ -5777,13 +5777,13 @@
       </c>
       <c r="C108" s="29" t="inlineStr">
         <is>
-          <t>PCB alimentación: diseño esquemático [8 HH]</t>
+          <t>Upload concurrente con adquisicion: sensor_task adquiere mientras modem sube. Validado con TRIG_006/007/008 simultaneos. [4 HH]</t>
         </is>
       </c>
       <c r="D108" s="1" t="n"/>
       <c r="E108" s="29" t="inlineStr">
         <is>
-          <t>Monitoreo fotovoltaico</t>
+          <t>Modem_PowerOff: NRST residual posible por corriente</t>
         </is>
       </c>
       <c r="F108" s="29" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="H108" s="29" t="inlineStr">
         <is>
-          <t>Validación banco baterías Li-Ion: capacidad y ciclos [6 HH]</t>
+          <t>NTP: debug con dump AT completo + timing [4 HH]</t>
         </is>
       </c>
       <c r="I108" s="1" t="n"/>
@@ -5827,7 +5827,7 @@
       </c>
       <c r="C109" s="29" t="inlineStr">
         <is>
-          <t>Protecciones eléctricas: TVS + Polyswitch [4 HH]</t>
+          <t>GANTT actualizado. Documentacion de arquitectura. [2 HH]</t>
         </is>
       </c>
       <c r="D109" s="1" t="n"/>
@@ -5842,7 +5842,7 @@
       </c>
       <c r="H109" s="29" t="inlineStr">
         <is>
-          <t>PCB alimentación: layout y routing [10 HH]</t>
+          <t>Documentacion tecnica v1.2.0 + GANTT final [2 HH]</t>
         </is>
       </c>
       <c r="I109" s="1" t="n"/>

</xml_diff>

<commit_message>
fix: planning row heights for Jun+ weeks (13px->45px)
</commit_message>
<xml_diff>
--- a/docs/planning/creador gantt/Planificación semanal actual .xlsx
+++ b/docs/planning/creador gantt/Planificación semanal actual .xlsx
@@ -4290,7 +4290,7 @@
       <c r="AA75" s="1" t="n"/>
       <c r="AB75" s="1" t="n"/>
     </row>
-    <row r="76" ht="13" customHeight="1" s="25">
+    <row r="76" ht="15" customHeight="1" s="25">
       <c r="A76" s="1" t="n"/>
       <c r="B76" s="27" t="inlineStr">
         <is>
@@ -4324,7 +4324,7 @@
       <c r="AA76" s="1" t="n"/>
       <c r="AB76" s="1" t="n"/>
     </row>
-    <row r="77" ht="13" customHeight="1" s="25">
+    <row r="77" ht="15" customHeight="1" s="25">
       <c r="A77" s="1" t="n"/>
       <c r="B77" s="28" t="inlineStr">
         <is>
@@ -4390,7 +4390,7 @@
       <c r="AA77" s="1" t="n"/>
       <c r="AB77" s="1" t="n"/>
     </row>
-    <row r="78" ht="13" customHeight="1" s="25">
+    <row r="78" ht="45" customHeight="1" s="25">
       <c r="A78" s="1" t="n"/>
       <c r="B78" s="1" t="n">
         <v>1</v>
@@ -4436,7 +4436,7 @@
       <c r="AA78" s="1" t="n"/>
       <c r="AB78" s="1" t="n"/>
     </row>
-    <row r="79" ht="13" customHeight="1" s="25">
+    <row r="79" ht="45" customHeight="1" s="25">
       <c r="A79" s="1" t="n"/>
       <c r="B79" s="1" t="n">
         <v>2</v>
@@ -4482,7 +4482,7 @@
       <c r="AA79" s="1" t="n"/>
       <c r="AB79" s="1" t="n"/>
     </row>
-    <row r="80" ht="13" customHeight="1" s="25">
+    <row r="80" ht="45" customHeight="1" s="25">
       <c r="A80" s="1" t="n"/>
       <c r="B80" s="1" t="n">
         <v>3</v>
@@ -4528,7 +4528,7 @@
       <c r="AA80" s="1" t="n"/>
       <c r="AB80" s="1" t="n"/>
     </row>
-    <row r="81" ht="13" customHeight="1" s="25">
+    <row r="81" ht="45" customHeight="1" s="25">
       <c r="A81" s="1" t="n"/>
       <c r="B81" s="1" t="n">
         <v>4</v>
@@ -4611,7 +4611,7 @@
       <c r="AA82" s="1" t="n"/>
       <c r="AB82" s="1" t="n"/>
     </row>
-    <row r="83" ht="13" customHeight="1" s="25">
+    <row r="83" ht="15" customHeight="1" s="25">
       <c r="A83" s="1" t="n"/>
       <c r="B83" s="27" t="inlineStr">
         <is>
@@ -4645,7 +4645,7 @@
       <c r="AA83" s="1" t="n"/>
       <c r="AB83" s="1" t="n"/>
     </row>
-    <row r="84" ht="13" customHeight="1" s="25">
+    <row r="84" ht="15" customHeight="1" s="25">
       <c r="A84" s="1" t="n"/>
       <c r="B84" s="28" t="inlineStr">
         <is>
@@ -4711,7 +4711,7 @@
       <c r="AA84" s="1" t="n"/>
       <c r="AB84" s="1" t="n"/>
     </row>
-    <row r="85" ht="13" customHeight="1" s="25">
+    <row r="85" ht="45" customHeight="1" s="25">
       <c r="A85" s="1" t="n"/>
       <c r="B85" s="1" t="n">
         <v>1</v>
@@ -4757,7 +4757,7 @@
       <c r="AA85" s="1" t="n"/>
       <c r="AB85" s="1" t="n"/>
     </row>
-    <row r="86" ht="13" customHeight="1" s="25">
+    <row r="86" ht="45" customHeight="1" s="25">
       <c r="A86" s="1" t="n"/>
       <c r="B86" s="1" t="n">
         <v>2</v>
@@ -4803,7 +4803,7 @@
       <c r="AA86" s="1" t="n"/>
       <c r="AB86" s="1" t="n"/>
     </row>
-    <row r="87" ht="13" customHeight="1" s="25">
+    <row r="87" ht="45" customHeight="1" s="25">
       <c r="A87" s="1" t="n"/>
       <c r="B87" s="1" t="n">
         <v>3</v>
@@ -4845,7 +4845,7 @@
       <c r="AA87" s="1" t="n"/>
       <c r="AB87" s="1" t="n"/>
     </row>
-    <row r="88" ht="13" customHeight="1" s="25">
+    <row r="88" ht="45" customHeight="1" s="25">
       <c r="A88" s="1" t="n"/>
       <c r="B88" s="1" t="n">
         <v>4</v>
@@ -4924,7 +4924,7 @@
       <c r="AA89" s="1" t="n"/>
       <c r="AB89" s="1" t="n"/>
     </row>
-    <row r="90" ht="13" customHeight="1" s="25">
+    <row r="90" ht="15" customHeight="1" s="25">
       <c r="A90" s="1" t="n"/>
       <c r="B90" s="27" t="inlineStr">
         <is>
@@ -4958,7 +4958,7 @@
       <c r="AA90" s="1" t="n"/>
       <c r="AB90" s="1" t="n"/>
     </row>
-    <row r="91" ht="13" customHeight="1" s="25">
+    <row r="91" ht="15" customHeight="1" s="25">
       <c r="A91" s="1" t="n"/>
       <c r="B91" s="28" t="inlineStr">
         <is>
@@ -5024,7 +5024,7 @@
       <c r="AA91" s="1" t="n"/>
       <c r="AB91" s="1" t="n"/>
     </row>
-    <row r="92" ht="13" customHeight="1" s="25">
+    <row r="92" ht="45" customHeight="1" s="25">
       <c r="A92" s="1" t="n"/>
       <c r="B92" s="1" t="n">
         <v>1</v>
@@ -5070,7 +5070,7 @@
       <c r="AA92" s="1" t="n"/>
       <c r="AB92" s="1" t="n"/>
     </row>
-    <row r="93" ht="13" customHeight="1" s="25">
+    <row r="93" ht="45" customHeight="1" s="25">
       <c r="A93" s="1" t="n"/>
       <c r="B93" s="1" t="n">
         <v>2</v>
@@ -5116,7 +5116,7 @@
       <c r="AA93" s="1" t="n"/>
       <c r="AB93" s="1" t="n"/>
     </row>
-    <row r="94" ht="13" customHeight="1" s="25">
+    <row r="94" ht="45" customHeight="1" s="25">
       <c r="A94" s="1" t="n"/>
       <c r="B94" s="1" t="n">
         <v>3</v>
@@ -5158,7 +5158,7 @@
       <c r="AA94" s="1" t="n"/>
       <c r="AB94" s="1" t="n"/>
     </row>
-    <row r="95" ht="13" customHeight="1" s="25">
+    <row r="95" ht="45" customHeight="1" s="25">
       <c r="A95" s="1" t="n"/>
       <c r="B95" s="1" t="n">
         <v>4</v>
@@ -5237,7 +5237,7 @@
       <c r="AA96" s="1" t="n"/>
       <c r="AB96" s="1" t="n"/>
     </row>
-    <row r="97" ht="13" customHeight="1" s="25">
+    <row r="97" ht="15" customHeight="1" s="25">
       <c r="A97" s="1" t="n"/>
       <c r="B97" s="27" t="inlineStr">
         <is>
@@ -5271,7 +5271,7 @@
       <c r="AA97" s="1" t="n"/>
       <c r="AB97" s="1" t="n"/>
     </row>
-    <row r="98" ht="13" customHeight="1" s="25">
+    <row r="98" ht="15" customHeight="1" s="25">
       <c r="A98" s="1" t="n"/>
       <c r="B98" s="28" t="inlineStr">
         <is>
@@ -5337,7 +5337,7 @@
       <c r="AA98" s="1" t="n"/>
       <c r="AB98" s="1" t="n"/>
     </row>
-    <row r="99" ht="13" customHeight="1" s="25">
+    <row r="99" ht="45" customHeight="1" s="25">
       <c r="A99" s="1" t="n"/>
       <c r="B99" s="1" t="n">
         <v>1</v>
@@ -5387,7 +5387,7 @@
       <c r="AA99" s="1" t="n"/>
       <c r="AB99" s="1" t="n"/>
     </row>
-    <row r="100" ht="13" customHeight="1" s="25">
+    <row r="100" ht="45" customHeight="1" s="25">
       <c r="A100" s="1" t="n"/>
       <c r="B100" s="1" t="n">
         <v>2</v>
@@ -5437,7 +5437,7 @@
       <c r="AA100" s="1" t="n"/>
       <c r="AB100" s="1" t="n"/>
     </row>
-    <row r="101" ht="13" customHeight="1" s="25">
+    <row r="101" ht="45" customHeight="1" s="25">
       <c r="A101" s="1" t="n"/>
       <c r="B101" s="1" t="n">
         <v>3</v>
@@ -5487,7 +5487,7 @@
       <c r="AA101" s="1" t="n"/>
       <c r="AB101" s="1" t="n"/>
     </row>
-    <row r="102" ht="13" customHeight="1" s="25">
+    <row r="102" ht="45" customHeight="1" s="25">
       <c r="A102" s="1" t="n"/>
       <c r="B102" s="1" t="n">
         <v>4</v>
@@ -5570,7 +5570,7 @@
       <c r="AA103" s="1" t="n"/>
       <c r="AB103" s="1" t="n"/>
     </row>
-    <row r="104" ht="13" customHeight="1" s="25">
+    <row r="104" ht="15" customHeight="1" s="25">
       <c r="A104" s="1" t="n"/>
       <c r="B104" s="27" t="inlineStr">
         <is>
@@ -5604,7 +5604,7 @@
       <c r="AA104" s="1" t="n"/>
       <c r="AB104" s="1" t="n"/>
     </row>
-    <row r="105" ht="13" customHeight="1" s="25">
+    <row r="105" ht="15" customHeight="1" s="25">
       <c r="A105" s="1" t="n"/>
       <c r="B105" s="28" t="inlineStr">
         <is>
@@ -5670,7 +5670,7 @@
       <c r="AA105" s="1" t="n"/>
       <c r="AB105" s="1" t="n"/>
     </row>
-    <row r="106" ht="13" customHeight="1" s="25">
+    <row r="106" ht="45" customHeight="1" s="25">
       <c r="A106" s="1" t="n"/>
       <c r="B106" s="1" t="n">
         <v>1</v>
@@ -5720,7 +5720,7 @@
       <c r="AA106" s="1" t="n"/>
       <c r="AB106" s="1" t="n"/>
     </row>
-    <row r="107" ht="13" customHeight="1" s="25">
+    <row r="107" ht="45" customHeight="1" s="25">
       <c r="A107" s="1" t="n"/>
       <c r="B107" s="1" t="n">
         <v>2</v>
@@ -5770,7 +5770,7 @@
       <c r="AA107" s="1" t="n"/>
       <c r="AB107" s="1" t="n"/>
     </row>
-    <row r="108" ht="13" customHeight="1" s="25">
+    <row r="108" ht="45" customHeight="1" s="25">
       <c r="A108" s="1" t="n"/>
       <c r="B108" s="1" t="n">
         <v>3</v>
@@ -5820,7 +5820,7 @@
       <c r="AA108" s="1" t="n"/>
       <c r="AB108" s="1" t="n"/>
     </row>
-    <row r="109" ht="13" customHeight="1" s="25">
+    <row r="109" ht="45" customHeight="1" s="25">
       <c r="A109" s="1" t="n"/>
       <c r="B109" s="1" t="n">
         <v>4</v>
@@ -5903,7 +5903,7 @@
       <c r="AA110" s="1" t="n"/>
       <c r="AB110" s="1" t="n"/>
     </row>
-    <row r="111" ht="13" customHeight="1" s="25">
+    <row r="111" ht="15" customHeight="1" s="25">
       <c r="A111" s="1" t="n"/>
       <c r="B111" s="27" t="inlineStr">
         <is>
@@ -5937,7 +5937,7 @@
       <c r="AA111" s="1" t="n"/>
       <c r="AB111" s="1" t="n"/>
     </row>
-    <row r="112" ht="13" customHeight="1" s="25">
+    <row r="112" ht="15" customHeight="1" s="25">
       <c r="A112" s="1" t="n"/>
       <c r="B112" s="28" t="inlineStr">
         <is>
@@ -6003,7 +6003,7 @@
       <c r="AA112" s="1" t="n"/>
       <c r="AB112" s="1" t="n"/>
     </row>
-    <row r="113" ht="13" customHeight="1" s="25">
+    <row r="113" ht="45" customHeight="1" s="25">
       <c r="A113" s="1" t="n"/>
       <c r="B113" s="1" t="n">
         <v>1</v>
@@ -6049,7 +6049,7 @@
       <c r="AA113" s="1" t="n"/>
       <c r="AB113" s="1" t="n"/>
     </row>
-    <row r="114" ht="13" customHeight="1" s="25">
+    <row r="114" ht="45" customHeight="1" s="25">
       <c r="A114" s="1" t="n"/>
       <c r="B114" s="1" t="n">
         <v>2</v>
@@ -6095,7 +6095,7 @@
       <c r="AA114" s="1" t="n"/>
       <c r="AB114" s="1" t="n"/>
     </row>
-    <row r="115" ht="13" customHeight="1" s="25">
+    <row r="115" ht="45" customHeight="1" s="25">
       <c r="A115" s="1" t="n"/>
       <c r="B115" s="1" t="n">
         <v>3</v>
@@ -6141,7 +6141,7 @@
       <c r="AA115" s="1" t="n"/>
       <c r="AB115" s="1" t="n"/>
     </row>
-    <row r="116" ht="13" customHeight="1" s="25">
+    <row r="116" ht="45" customHeight="1" s="25">
       <c r="A116" s="1" t="n"/>
       <c r="B116" s="1" t="n">
         <v>4</v>
@@ -6220,7 +6220,7 @@
       <c r="AA117" s="1" t="n"/>
       <c r="AB117" s="1" t="n"/>
     </row>
-    <row r="118" ht="13" customHeight="1" s="25">
+    <row r="118" ht="15" customHeight="1" s="25">
       <c r="A118" s="1" t="n"/>
       <c r="B118" s="27" t="inlineStr">
         <is>
@@ -6254,7 +6254,7 @@
       <c r="AA118" s="1" t="n"/>
       <c r="AB118" s="1" t="n"/>
     </row>
-    <row r="119" ht="13" customHeight="1" s="25">
+    <row r="119" ht="15" customHeight="1" s="25">
       <c r="A119" s="1" t="n"/>
       <c r="B119" s="28" t="inlineStr">
         <is>
@@ -6320,7 +6320,7 @@
       <c r="AA119" s="1" t="n"/>
       <c r="AB119" s="1" t="n"/>
     </row>
-    <row r="120" ht="13" customHeight="1" s="25">
+    <row r="120" ht="45" customHeight="1" s="25">
       <c r="A120" s="1" t="n"/>
       <c r="B120" s="1" t="n">
         <v>1</v>
@@ -6366,7 +6366,7 @@
       <c r="AA120" s="1" t="n"/>
       <c r="AB120" s="1" t="n"/>
     </row>
-    <row r="121" ht="13" customHeight="1" s="25">
+    <row r="121" ht="45" customHeight="1" s="25">
       <c r="A121" s="1" t="n"/>
       <c r="B121" s="1" t="n">
         <v>2</v>
@@ -6412,7 +6412,7 @@
       <c r="AA121" s="1" t="n"/>
       <c r="AB121" s="1" t="n"/>
     </row>
-    <row r="122" ht="13" customHeight="1" s="25">
+    <row r="122" ht="45" customHeight="1" s="25">
       <c r="A122" s="1" t="n"/>
       <c r="B122" s="1" t="n">
         <v>3</v>
@@ -6458,7 +6458,7 @@
       <c r="AA122" s="1" t="n"/>
       <c r="AB122" s="1" t="n"/>
     </row>
-    <row r="123" ht="13" customHeight="1" s="25">
+    <row r="123" ht="45" customHeight="1" s="25">
       <c r="A123" s="1" t="n"/>
       <c r="B123" s="1" t="n">
         <v>4</v>
@@ -6537,7 +6537,7 @@
       <c r="AA124" s="1" t="n"/>
       <c r="AB124" s="1" t="n"/>
     </row>
-    <row r="125" ht="13" customHeight="1" s="25">
+    <row r="125" ht="15" customHeight="1" s="25">
       <c r="A125" s="1" t="n"/>
       <c r="B125" s="27" t="inlineStr">
         <is>
@@ -6571,7 +6571,7 @@
       <c r="AA125" s="1" t="n"/>
       <c r="AB125" s="1" t="n"/>
     </row>
-    <row r="126" ht="13" customHeight="1" s="25">
+    <row r="126" ht="15" customHeight="1" s="25">
       <c r="A126" s="1" t="n"/>
       <c r="B126" s="28" t="inlineStr">
         <is>
@@ -6637,7 +6637,7 @@
       <c r="AA126" s="1" t="n"/>
       <c r="AB126" s="1" t="n"/>
     </row>
-    <row r="127" ht="13" customHeight="1" s="25">
+    <row r="127" ht="45" customHeight="1" s="25">
       <c r="A127" s="1" t="n"/>
       <c r="B127" s="1" t="n">
         <v>1</v>
@@ -6683,7 +6683,7 @@
       <c r="AA127" s="1" t="n"/>
       <c r="AB127" s="1" t="n"/>
     </row>
-    <row r="128" ht="13" customHeight="1" s="25">
+    <row r="128" ht="45" customHeight="1" s="25">
       <c r="A128" s="1" t="n"/>
       <c r="B128" s="1" t="n">
         <v>2</v>
@@ -6729,7 +6729,7 @@
       <c r="AA128" s="1" t="n"/>
       <c r="AB128" s="1" t="n"/>
     </row>
-    <row r="129" ht="13" customHeight="1" s="25">
+    <row r="129" ht="45" customHeight="1" s="25">
       <c r="A129" s="1" t="n"/>
       <c r="B129" s="1" t="n">
         <v>3</v>
@@ -6775,7 +6775,7 @@
       <c r="AA129" s="1" t="n"/>
       <c r="AB129" s="1" t="n"/>
     </row>
-    <row r="130" ht="13" customHeight="1" s="25">
+    <row r="130" ht="45" customHeight="1" s="25">
       <c r="A130" s="1" t="n"/>
       <c r="B130" s="1" t="n">
         <v>4</v>
@@ -6884,7 +6884,7 @@
       <c r="AA132" s="1" t="n"/>
       <c r="AB132" s="1" t="n"/>
     </row>
-    <row r="133" ht="13" customHeight="1" s="25">
+    <row r="133" ht="15" customHeight="1" s="25">
       <c r="A133" s="1" t="n"/>
       <c r="B133" s="31" t="inlineStr">
         <is>

</xml_diff>